<commit_message>
Alterações na lição 3 do S3
</commit_message>
<xml_diff>
--- a/Files/P1/S3_MOOC_Template_Grupo1.xlsx
+++ b/Files/P1/S3_MOOC_Template_Grupo1.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\CAMUL\CAMUL-2026\Files\P1\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Games\GameDevProjects\CAMUL-2026\Files\P1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{189E0B39-FB07-4E72-97FE-C2776E7AFE9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B63F109D-1B36-46F9-80E4-4B67AEBCF4C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Enquadramento" sheetId="1" r:id="rId1"/>
@@ -178,40 +178,10 @@
 Tag laranja no telefone: rede de 3 contactos e substituto.</t>
   </si>
   <si>
-    <t>Lição 3: Primeiro contacto — acalmar</t>
-  </si>
-  <si>
-    <t>No fim da lição, o cuidador é capaz de:
-• identificar sinais de angústia na pessoa com demência;
-• aplicar técnicas para a acalmar (aproximação calma, frases curtas, validar, reduzir estímulos);
-• usar uma técnica rápida de autorregulação antes de intervir («acalmar-se para acalmar»).</t>
-  </si>
-  <si>
     <t>Vídeo (dramatização certo vs. errado)</t>
   </si>
   <si>
-    <t>Pessoa: observar sinais (inquietação, choro, querer ir embora, recusa); aproximar-se de frente e devagar; uma ideia por frase; validar emoções em vez de corrigir; reduzir ruído e movimento; objetos de conforto.
-Cuidador: respiração lenta, pausa de 10 segundos, pedir a outra pessoa que assuma por instantes.</t>
-  </si>
-  <si>
     <t>Dramatização com 2 atores: a mesma cena feita da forma errada e da forma certa; narração aponta as diferenças.</t>
-  </si>
-  <si>
-    <t>Storyboard: (1) D. Rosa agitada no momento da evacuação/confinamento → (2) versão errada (pressa, contrariar) → (3) pausa: Ana respira → (4) versão certa → (5) resumo das técnicas.
-Recursos: atores, guião de diálogo, legendas.</t>
-  </si>
-  <si>
-    <t>Abertura: «Quando a pessoa com demência entra em pânico, as palavras contam menos do que o tom. E o tom começa na sua própria calma.»</t>
-  </si>
-  <si>
-    <t>OMS (2011) Psychological First Aid: Guide for Field Workers
-ADI (2022) conselhos de comunicação em crise
-Alzheimer's Association — In a Disaster</t>
-  </si>
-  <si>
-    <t>Quiz de cenários: «O que dizias/fazias?» com feedback em cada opção (4 situações).
-Exercício: praticar a técnica de respiração guiada (1 min).
-Visita 3D (opcional): «Para onde levaria a D. Rosa e o que desligaria?» (resposta no quiz).</t>
   </si>
   <si>
     <t>Responsável: Rodrigo Silva
@@ -364,6 +334,43 @@
   </si>
   <si>
     <t>Udemy (≥ 30 min de vídeo, ≥ 5 aulas, vídeo HD 1080p, grátis abaixo de 2 h, quizzes nativos, revisão de qualidade antes de publicar; Matterport por link + vídeo gravado, sem iframe).</t>
+  </si>
+  <si>
+    <t>Lição 3: Primeiro contacto — acalmar (e acalmar-se)</t>
+  </si>
+  <si>
+    <t>No fim da lição, o cuidador é capaz de:
+• identificar sinais de angústia na pessoa com demência;
+• aplicar técnicas para a acalmar (aproximação calma, frases curtas, validar, reduzir estímulos);
+• executar uma técnica rápida de autorregulação («acalmar-se para acalmar»).</t>
+  </si>
+  <si>
+    <t>Pessoa: observar sinais (inquietação, choro, querer ir embora, recusa); aproximar-se de frente e devagar; uma ideia por frase; validar emoções em vez de corrigir; reduzir estimulos; reconfortar.
+Cuidador: respiração lenta, pausa de 10 segundos, pedir a outra pessoa que assuma por instantes.</t>
+  </si>
+  <si>
+    <t>Storyboard: (1) Doente agitado no momento da evacuação/confinamento → (2) versão errada (pressa, contrariar) → (3) pausa: Cuidador respira → (4) versão certa (aproxima-se de frente, desliga a TV) → (5) resumo das técnicas.
+Recursos: atores, guião de diálogo, legendas.</t>
+  </si>
+  <si>
+    <t>Abertura: «Quando a pessoa com demência entra em pânico, as palavras contam menos do que o tom. E o tom começa na sua própria calma.»
+Versão Errada: Cuidador «Temos de sair já! Pare de chorar não há tempo!» Doente«Não vou! Quero ir para casa!» Cuidador «Mas já está em casa!»
+Narração: «Pressa, voz alta e contrariar só aumentam o medo.»
+Versão certa: Cuidador respira, aproxima-se de frente: «(Nome do doente), sou o/a (Nome do cuidador). Estou aqui consigo.» «Está assustado. Eu percebo.» «Vamos juntos.» (desliga a TV)
+Fecho: «Respire, aproxime-se, reduza, acolha, reconforte. Na próxima lição, vemos como ajudar a pessoa a sair em segurança.»</t>
+  </si>
+  <si>
+    <t>Respiração Guiada
+Quiz de cenários: «O que dizias/fazias?» com feedback em cada opção (4 situações).
+Exercício: praticar a técnica de respiração guiada (1 min).
+Visita 3D (opcional): «Para onde levaria o Doente e o que desligaria?» (resposta no quiz).</t>
+  </si>
+  <si>
+    <t>OMS (2011) Psychological First Aid: Guide for Field Workers
+ADI (2022) conselhos de comunicação em crise
+Alzheimer's Association — In a Disaster
+Alzheimer Portugal (2025) Estratégias de Comunicação com a Pessoa com Demência
+Ordem dos Psicólogos Portugueses (2015), Intervenção Psicológica em Crise e Catástrofe</t>
   </si>
 </sst>
 </file>
@@ -806,90 +813,90 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B10"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
     <col min="2" max="2" width="110" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="13" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="B1" s="14" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="36" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="13" t="s">
+        <v>63</v>
+      </c>
+      <c r="B2" s="14" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="B3" s="14" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" ht="54" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="13" t="s">
+        <v>66</v>
+      </c>
+      <c r="B4" s="14" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="13" t="s">
+        <v>67</v>
+      </c>
+      <c r="B5" s="14" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" ht="54" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="13" t="s">
+        <v>69</v>
+      </c>
+      <c r="B6" s="14" t="s">
         <v>70</v>
       </c>
-      <c r="B2" s="14" t="s">
+    </row>
+    <row r="7" spans="1:2" ht="90" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="13" t="s">
         <v>71</v>
       </c>
-    </row>
-    <row r="3" spans="1:2" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="13" t="s">
+      <c r="B7" s="14" t="s">
         <v>72</v>
       </c>
-      <c r="B3" s="14" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" ht="54" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="13" t="s">
+    </row>
+    <row r="8" spans="1:2" ht="54" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="13" t="s">
         <v>73</v>
       </c>
-      <c r="B4" s="14" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="13" t="s">
+      <c r="B8" s="14" t="s">
         <v>74</v>
       </c>
-      <c r="B5" s="14" t="s">
+    </row>
+    <row r="9" spans="1:2" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="13" t="s">
         <v>75</v>
       </c>
-    </row>
-    <row r="6" spans="1:2" ht="54" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="13" t="s">
+      <c r="B9" s="14" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" ht="90" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="13" t="s">
         <v>76</v>
       </c>
-      <c r="B6" s="14" t="s">
+      <c r="B10" s="14" t="s">
         <v>77</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" ht="90" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="13" t="s">
-        <v>78</v>
-      </c>
-      <c r="B7" s="14" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" ht="54" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="13" t="s">
-        <v>80</v>
-      </c>
-      <c r="B8" s="14" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="13" t="s">
-        <v>82</v>
-      </c>
-      <c r="B9" s="14" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" ht="90" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="13" t="s">
-        <v>83</v>
-      </c>
-      <c r="B10" s="14" t="s">
-        <v>84</v>
       </c>
     </row>
   </sheetData>
@@ -900,26 +907,26 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:O62"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="41.5546875" customWidth="1"/>
-    <col min="2" max="2" width="16.21875" customWidth="1"/>
-    <col min="3" max="3" width="43.5546875" customWidth="1"/>
-    <col min="4" max="4" width="26.21875" customWidth="1"/>
-    <col min="5" max="5" width="14.5546875" customWidth="1"/>
+    <col min="1" max="1" width="41.5703125" customWidth="1"/>
+    <col min="2" max="2" width="16.28515625" customWidth="1"/>
+    <col min="3" max="3" width="43.5703125" customWidth="1"/>
+    <col min="4" max="4" width="26.28515625" customWidth="1"/>
+    <col min="5" max="5" width="14.5703125" customWidth="1"/>
     <col min="6" max="6" width="41" customWidth="1"/>
-    <col min="7" max="7" width="38.44140625" customWidth="1"/>
-    <col min="8" max="8" width="23.88671875" customWidth="1"/>
-    <col min="9" max="9" width="37.77734375" customWidth="1"/>
-    <col min="10" max="10" width="39.6640625" customWidth="1"/>
-    <col min="11" max="11" width="36.109375" customWidth="1"/>
-    <col min="12" max="12" width="41.6640625" customWidth="1"/>
-    <col min="13" max="13" width="29.88671875" customWidth="1"/>
+    <col min="7" max="7" width="38.42578125" customWidth="1"/>
+    <col min="8" max="8" width="23.85546875" customWidth="1"/>
+    <col min="9" max="9" width="37.7109375" customWidth="1"/>
+    <col min="10" max="10" width="39.7109375" customWidth="1"/>
+    <col min="11" max="11" width="36.140625" customWidth="1"/>
+    <col min="12" max="12" width="41.7109375" customWidth="1"/>
+    <col min="13" max="13" width="29.85546875" customWidth="1"/>
     <col min="14" max="14" width="52" customWidth="1"/>
     <col min="15" max="15" width="60" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" ht="72" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:15" ht="72" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -966,7 +973,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="2" spans="1:15" ht="240" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:15" ht="240" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="18" t="s">
         <v>15</v>
       </c>
@@ -1013,7 +1020,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="3" spans="1:15" ht="240" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:15" ht="240" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="17"/>
       <c r="B3" s="17"/>
       <c r="C3" s="15" t="s">
@@ -1056,11 +1063,11 @@
         <v>38</v>
       </c>
     </row>
-    <row r="4" spans="1:15" ht="240" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:15" ht="299.25" x14ac:dyDescent="0.25">
       <c r="A4" s="17"/>
       <c r="B4" s="17"/>
       <c r="C4" s="15" t="s">
-        <v>39</v>
+        <v>81</v>
       </c>
       <c r="D4" s="14" t="s">
         <v>16</v>
@@ -1069,41 +1076,41 @@
         <v>18</v>
       </c>
       <c r="F4" s="14" t="s">
-        <v>40</v>
+        <v>82</v>
       </c>
       <c r="G4" s="14" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="H4" s="14" t="s">
         <v>21</v>
       </c>
       <c r="I4" s="14" t="s">
-        <v>42</v>
+        <v>83</v>
       </c>
       <c r="J4" s="14" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="K4" s="14" t="s">
-        <v>44</v>
+        <v>84</v>
       </c>
       <c r="L4" s="14" t="s">
-        <v>45</v>
+        <v>85</v>
       </c>
       <c r="M4" s="14" t="s">
-        <v>46</v>
+        <v>87</v>
       </c>
       <c r="N4" s="14" t="s">
-        <v>47</v>
+        <v>86</v>
       </c>
       <c r="O4" s="14" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="5" spans="1:15" ht="240" customHeight="1" x14ac:dyDescent="0.3">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" ht="240" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="17"/>
       <c r="B5" s="17"/>
       <c r="C5" s="15" t="s">
-        <v>49</v>
+        <v>42</v>
       </c>
       <c r="D5" s="14" t="s">
         <v>16</v>
@@ -1112,41 +1119,41 @@
         <v>18</v>
       </c>
       <c r="F5" s="14" t="s">
-        <v>50</v>
+        <v>43</v>
       </c>
       <c r="G5" s="14" t="s">
-        <v>51</v>
+        <v>44</v>
       </c>
       <c r="H5" s="14" t="s">
         <v>21</v>
       </c>
       <c r="I5" s="14" t="s">
-        <v>52</v>
+        <v>45</v>
       </c>
       <c r="J5" s="14" t="s">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="K5" s="14" t="s">
-        <v>54</v>
+        <v>47</v>
       </c>
       <c r="L5" s="14" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="M5" s="14" t="s">
-        <v>56</v>
+        <v>49</v>
       </c>
       <c r="N5" s="14" t="s">
-        <v>57</v>
+        <v>50</v>
       </c>
       <c r="O5" s="14" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="6" spans="1:15" ht="240" customHeight="1" x14ac:dyDescent="0.3">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" ht="240" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="17"/>
       <c r="B6" s="17"/>
       <c r="C6" s="15" t="s">
-        <v>59</v>
+        <v>52</v>
       </c>
       <c r="D6" s="14" t="s">
         <v>16</v>
@@ -1155,37 +1162,37 @@
         <v>18</v>
       </c>
       <c r="F6" s="14" t="s">
-        <v>60</v>
+        <v>53</v>
       </c>
       <c r="G6" s="14" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="H6" s="14" t="s">
         <v>21</v>
       </c>
       <c r="I6" s="14" t="s">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="J6" s="14" t="s">
-        <v>63</v>
+        <v>56</v>
       </c>
       <c r="K6" s="14" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="L6" s="14" t="s">
-        <v>65</v>
+        <v>58</v>
       </c>
       <c r="M6" s="14" t="s">
-        <v>66</v>
+        <v>59</v>
       </c>
       <c r="N6" s="14" t="s">
-        <v>67</v>
+        <v>60</v>
       </c>
       <c r="O6" s="14" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="7" spans="1:15" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="6"/>
       <c r="B7" s="4"/>
       <c r="D7" s="4"/>
@@ -1201,7 +1208,7 @@
       <c r="N7" s="4"/>
       <c r="O7" s="4"/>
     </row>
-    <row r="8" spans="1:15" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:15" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="6"/>
       <c r="B8" s="4"/>
       <c r="C8" s="4"/>
@@ -1218,7 +1225,7 @@
       <c r="N8" s="5"/>
       <c r="O8" s="4"/>
     </row>
-    <row r="9" spans="1:15" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:15" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="3"/>
       <c r="B9" s="4"/>
       <c r="C9" s="4"/>
@@ -1234,7 +1241,7 @@
       <c r="N9" s="5"/>
       <c r="O9" s="4"/>
     </row>
-    <row r="10" spans="1:15" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:15" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="6"/>
       <c r="B10" s="4"/>
       <c r="C10" s="4"/>
@@ -1251,7 +1258,7 @@
       <c r="N10" s="5"/>
       <c r="O10" s="4"/>
     </row>
-    <row r="11" spans="1:15" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:15" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="6"/>
       <c r="B11" s="4"/>
       <c r="C11" s="4"/>
@@ -1268,7 +1275,7 @@
       <c r="N11" s="5"/>
       <c r="O11" s="4"/>
     </row>
-    <row r="12" spans="1:15" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:15" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="6"/>
       <c r="B12" s="4"/>
       <c r="D12" s="4"/>
@@ -1283,7 +1290,7 @@
       <c r="N12" s="5"/>
       <c r="O12" s="4"/>
     </row>
-    <row r="13" spans="1:15" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:15" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="6"/>
       <c r="B13" s="4"/>
       <c r="D13" s="4"/>
@@ -1298,7 +1305,7 @@
       <c r="N13" s="5"/>
       <c r="O13" s="4"/>
     </row>
-    <row r="14" spans="1:15" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:15" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="6"/>
       <c r="B14" s="4"/>
       <c r="D14" s="4"/>
@@ -1314,7 +1321,7 @@
       <c r="N14" s="5"/>
       <c r="O14" s="4"/>
     </row>
-    <row r="15" spans="1:15" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:15" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="6"/>
       <c r="B15" s="4"/>
       <c r="D15" s="4"/>
@@ -1329,7 +1336,7 @@
       <c r="N15" s="5"/>
       <c r="O15" s="4"/>
     </row>
-    <row r="16" spans="1:15" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:15" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="6"/>
       <c r="B16" s="4"/>
       <c r="C16" s="4"/>
@@ -1344,7 +1351,7 @@
       <c r="N16" s="5"/>
       <c r="O16" s="4"/>
     </row>
-    <row r="17" spans="1:15" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:15" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="6"/>
       <c r="B17" s="4"/>
       <c r="C17" s="4"/>
@@ -1359,7 +1366,7 @@
       <c r="N17" s="5"/>
       <c r="O17" s="4"/>
     </row>
-    <row r="18" spans="1:15" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:15" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="3"/>
       <c r="B18" s="4"/>
       <c r="C18" s="4"/>
@@ -1375,7 +1382,7 @@
       <c r="N18" s="5"/>
       <c r="O18" s="4"/>
     </row>
-    <row r="19" spans="1:15" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:15" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="3"/>
       <c r="B19" s="4"/>
       <c r="C19" s="4"/>
@@ -1392,7 +1399,7 @@
       <c r="N19" s="5"/>
       <c r="O19" s="4"/>
     </row>
-    <row r="20" spans="1:15" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:15" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="3"/>
       <c r="B20" s="4"/>
       <c r="D20" s="4"/>
@@ -1408,7 +1415,7 @@
       <c r="N20" s="5"/>
       <c r="O20" s="4"/>
     </row>
-    <row r="21" spans="1:15" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:15" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="3"/>
       <c r="B21" s="4"/>
       <c r="C21" s="4"/>
@@ -1425,7 +1432,7 @@
       <c r="N21" s="5"/>
       <c r="O21" s="4"/>
     </row>
-    <row r="22" spans="1:15" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:15" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="3"/>
       <c r="B22" s="4"/>
       <c r="C22" s="4"/>
@@ -1442,7 +1449,7 @@
       <c r="N22" s="5"/>
       <c r="O22" s="4"/>
     </row>
-    <row r="23" spans="1:15" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:15" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="3"/>
       <c r="B23" s="4"/>
       <c r="C23" s="4"/>
@@ -1459,7 +1466,7 @@
       <c r="N23" s="5"/>
       <c r="O23" s="4"/>
     </row>
-    <row r="24" spans="1:15" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:15" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="3"/>
       <c r="B24" s="4"/>
       <c r="D24" s="4"/>
@@ -1475,7 +1482,7 @@
       <c r="N24" s="5"/>
       <c r="O24" s="4"/>
     </row>
-    <row r="25" spans="1:15" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:15" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="6"/>
       <c r="B25" s="4"/>
       <c r="C25" s="4"/>
@@ -1492,7 +1499,7 @@
       <c r="N25" s="5"/>
       <c r="O25" s="4"/>
     </row>
-    <row r="26" spans="1:15" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:15" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="6"/>
       <c r="B26" s="4"/>
       <c r="C26" s="4"/>
@@ -1507,7 +1514,7 @@
       <c r="N26" s="5"/>
       <c r="O26" s="4"/>
     </row>
-    <row r="27" spans="1:15" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:15" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="6"/>
       <c r="B27" s="4"/>
       <c r="C27" s="4"/>
@@ -1523,7 +1530,7 @@
       <c r="N27" s="5"/>
       <c r="O27" s="4"/>
     </row>
-    <row r="28" spans="1:15" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:15" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="3"/>
       <c r="D28" s="4"/>
       <c r="E28" s="4"/>
@@ -1538,7 +1545,7 @@
       <c r="N28" s="5"/>
       <c r="O28" s="4"/>
     </row>
-    <row r="29" spans="1:15" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:15" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="6"/>
       <c r="B29" s="4"/>
       <c r="D29" s="4"/>
@@ -1554,7 +1561,7 @@
       <c r="N29" s="5"/>
       <c r="O29" s="4"/>
     </row>
-    <row r="30" spans="1:15" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:15" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="6"/>
       <c r="B30" s="4"/>
       <c r="D30" s="4"/>
@@ -1570,7 +1577,7 @@
       <c r="N30" s="5"/>
       <c r="O30" s="4"/>
     </row>
-    <row r="31" spans="1:15" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:15" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="6"/>
       <c r="B31" s="4"/>
       <c r="D31" s="4"/>
@@ -1586,7 +1593,7 @@
       <c r="N31" s="5"/>
       <c r="O31" s="4"/>
     </row>
-    <row r="32" spans="1:15" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:15" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="6"/>
       <c r="B32" s="4"/>
       <c r="D32" s="4"/>
@@ -1602,7 +1609,7 @@
       <c r="N32" s="5"/>
       <c r="O32" s="4"/>
     </row>
-    <row r="33" spans="1:15" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:15" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="6"/>
       <c r="B33" s="4"/>
       <c r="D33" s="4"/>
@@ -1618,7 +1625,7 @@
       <c r="N33" s="5"/>
       <c r="O33" s="4"/>
     </row>
-    <row r="34" spans="1:15" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:15" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="6"/>
       <c r="B34" s="4"/>
       <c r="D34" s="4"/>
@@ -1633,7 +1640,7 @@
       <c r="N34" s="5"/>
       <c r="O34" s="4"/>
     </row>
-    <row r="35" spans="1:15" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:15" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="3"/>
       <c r="B35" s="4"/>
       <c r="D35" s="4"/>
@@ -1649,7 +1656,7 @@
       <c r="N35" s="5"/>
       <c r="O35" s="4"/>
     </row>
-    <row r="36" spans="1:15" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:15" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="6"/>
       <c r="B36" s="4"/>
       <c r="D36" s="4"/>
@@ -1665,7 +1672,7 @@
       <c r="N36" s="5"/>
       <c r="O36" s="4"/>
     </row>
-    <row r="37" spans="1:15" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:15" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="6"/>
       <c r="B37" s="4"/>
       <c r="D37" s="4"/>
@@ -1681,7 +1688,7 @@
       <c r="N37" s="5"/>
       <c r="O37" s="4"/>
     </row>
-    <row r="38" spans="1:15" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:15" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="6"/>
       <c r="B38" s="4"/>
       <c r="D38" s="4"/>
@@ -1697,7 +1704,7 @@
       <c r="N38" s="5"/>
       <c r="O38" s="4"/>
     </row>
-    <row r="39" spans="1:15" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:15" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="6"/>
       <c r="B39" s="4"/>
       <c r="D39" s="4"/>
@@ -1713,7 +1720,7 @@
       <c r="N39" s="5"/>
       <c r="O39" s="4"/>
     </row>
-    <row r="40" spans="1:15" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:15" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="6"/>
       <c r="B40" s="4"/>
       <c r="D40" s="4"/>
@@ -1729,7 +1736,7 @@
       <c r="N40" s="5"/>
       <c r="O40" s="4"/>
     </row>
-    <row r="41" spans="1:15" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:15" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="6"/>
       <c r="B41" s="4"/>
       <c r="D41" s="4"/>
@@ -1744,7 +1751,7 @@
       <c r="N41" s="5"/>
       <c r="O41" s="4"/>
     </row>
-    <row r="42" spans="1:15" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:15" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="3"/>
       <c r="B42" s="4"/>
       <c r="C42" s="4"/>
@@ -1756,7 +1763,7 @@
       <c r="I42" s="4"/>
       <c r="J42" s="4"/>
     </row>
-    <row r="43" spans="1:15" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:15" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="3"/>
       <c r="B43" s="4"/>
       <c r="C43" s="4"/>
@@ -1768,7 +1775,7 @@
       <c r="I43" s="4"/>
       <c r="J43" s="4"/>
     </row>
-    <row r="44" spans="1:15" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:15" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="3"/>
       <c r="B44" s="4"/>
       <c r="C44" s="4"/>
@@ -1784,7 +1791,7 @@
       <c r="M44" s="9"/>
       <c r="N44" s="9"/>
     </row>
-    <row r="45" spans="1:15" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:15" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="3"/>
       <c r="B45" s="4"/>
       <c r="C45" s="4"/>
@@ -1800,7 +1807,7 @@
       <c r="M45" s="9"/>
       <c r="N45" s="9"/>
     </row>
-    <row r="46" spans="1:15" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:15" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="3"/>
       <c r="B46" s="4"/>
       <c r="C46" s="4"/>
@@ -1812,7 +1819,7 @@
       <c r="I46" s="4"/>
       <c r="J46" s="4"/>
     </row>
-    <row r="47" spans="1:15" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:15" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="3"/>
       <c r="B47" s="4"/>
       <c r="C47" s="4"/>
@@ -1824,7 +1831,7 @@
       <c r="I47" s="4"/>
       <c r="J47" s="4"/>
     </row>
-    <row r="48" spans="1:15" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:15" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="3"/>
       <c r="B48" s="4"/>
       <c r="C48" s="8"/>
@@ -1836,7 +1843,7 @@
       <c r="I48" s="4"/>
       <c r="J48" s="4"/>
     </row>
-    <row r="49" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="3"/>
       <c r="B49" s="4"/>
       <c r="C49" s="4"/>
@@ -1848,7 +1855,7 @@
       <c r="I49" s="4"/>
       <c r="J49" s="4"/>
     </row>
-    <row r="50" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="3"/>
       <c r="B50" s="4"/>
       <c r="C50" s="4"/>
@@ -1860,7 +1867,7 @@
       <c r="I50" s="4"/>
       <c r="J50" s="4"/>
     </row>
-    <row r="51" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="3"/>
       <c r="B51" s="4"/>
       <c r="C51" s="4"/>
@@ -1872,7 +1879,7 @@
       <c r="I51" s="4"/>
       <c r="J51" s="4"/>
     </row>
-    <row r="52" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="3"/>
       <c r="B52" s="4"/>
       <c r="C52" s="4"/>
@@ -1884,7 +1891,7 @@
       <c r="I52" s="4"/>
       <c r="J52" s="4"/>
     </row>
-    <row r="53" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="3"/>
       <c r="B53" s="4"/>
       <c r="C53" s="4"/>
@@ -1896,7 +1903,7 @@
       <c r="I53" s="4"/>
       <c r="J53" s="4"/>
     </row>
-    <row r="54" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" s="3"/>
       <c r="B54" s="4"/>
       <c r="C54" s="4"/>
@@ -1908,7 +1915,7 @@
       <c r="I54" s="4"/>
       <c r="J54" s="4"/>
     </row>
-    <row r="55" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="3"/>
       <c r="B55" s="4"/>
       <c r="C55" s="4"/>
@@ -1920,7 +1927,7 @@
       <c r="I55" s="4"/>
       <c r="J55" s="4"/>
     </row>
-    <row r="56" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="3"/>
       <c r="B56" s="9"/>
       <c r="C56" s="10"/>
@@ -1932,38 +1939,38 @@
       <c r="I56" s="9"/>
       <c r="J56" s="9"/>
     </row>
-    <row r="57" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="11"/>
       <c r="C57" s="12"/>
       <c r="D57" s="4"/>
       <c r="F57" s="5"/>
       <c r="G57" s="4"/>
     </row>
-    <row r="58" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C58" s="12"/>
       <c r="D58" s="4"/>
       <c r="F58" s="5"/>
       <c r="G58" s="4"/>
     </row>
-    <row r="59" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C59" s="12"/>
       <c r="D59" s="4"/>
       <c r="F59" s="5"/>
       <c r="G59" s="4"/>
     </row>
-    <row r="60" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C60" s="12"/>
       <c r="D60" s="4"/>
       <c r="F60" s="5"/>
       <c r="G60" s="4"/>
     </row>
-    <row r="61" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C61" s="12"/>
       <c r="D61" s="4"/>
       <c r="F61" s="5"/>
       <c r="G61" s="4"/>
     </row>
-    <row r="62" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C62" s="4"/>
       <c r="D62" s="4"/>
       <c r="F62" s="5"/>

</xml_diff>

<commit_message>
Adicionado Estado da Arte aos documentos
</commit_message>
<xml_diff>
--- a/Files/P1/S3_MOOC_Template_Grupo1.xlsx
+++ b/Files/P1/S3_MOOC_Template_Grupo1.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Games\GameDevProjects\CAMUL-2026\Files\P1\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Desktop\Mestrado-Jogos\CAMUL\CAMUL-2026\Files\P1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B63F109D-1B36-46F9-80E4-4B67AEBCF4C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1EF87B56-DC2A-4D63-8C8A-F33009CE65EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Enquadramento" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="90">
   <si>
     <t xml:space="preserve">Chapter Title </t>
   </si>
@@ -371,6 +371,12 @@
 Alzheimer's Association — In a Disaster
 Alzheimer Portugal (2025) Estratégias de Comunicação com a Pessoa com Demência
 Ordem dos Psicólogos Portugueses (2015), Intervenção Psicológica em Crise e Catástrofe</t>
+  </si>
+  <si>
+    <t>Estado da arte</t>
+  </si>
+  <si>
+    <t>Já existem cursos sobre demência e cuidadores, mas são longos (23 sessões, 14 h a 51 h), gerais e centrados no dia a dia. Cada um tem algo de único: o iSupport (OMS) tem manual impresso e SMS para quem tem pouca literacia digital; o NAU junta vídeos, quizzes e manual de apoio; o da Tasmânia inclui testemunhos de pessoas com demência. Nas páginas consultadas, nenhum trata a crise, os PSP à dupla cuidador–pessoa com demência, nem oferece prática em 3D. Analisados: iSupport-Portugal (ICBAS-UP), NAU «Cuidadores Informais» (ESEP), Curso de Formação de Cuidadores (Santa Maria Saúde), iSupport (OMS), Understanding Dementia (Univ. da Tasmânia).</t>
   </si>
 </sst>
 </file>
@@ -488,7 +494,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -531,6 +537,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -812,14 +824,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
     <col min="2" max="2" width="110" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="13" t="s">
         <v>62</v>
       </c>
@@ -827,7 +839,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A2" s="13" t="s">
         <v>63</v>
       </c>
@@ -835,7 +847,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A3" s="13" t="s">
         <v>65</v>
       </c>
@@ -843,7 +855,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="54" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A4" s="13" t="s">
         <v>66</v>
       </c>
@@ -851,7 +863,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="5" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A5" s="13" t="s">
         <v>67</v>
       </c>
@@ -859,7 +871,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="6" spans="1:2" ht="54" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A6" s="13" t="s">
         <v>69</v>
       </c>
@@ -867,35 +879,43 @@
         <v>70</v>
       </c>
     </row>
-    <row r="7" spans="1:2" ht="90" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="13" t="s">
+    <row r="7" spans="1:2" ht="94.5" x14ac:dyDescent="0.25">
+      <c r="A7" s="19" t="s">
+        <v>88</v>
+      </c>
+      <c r="B7" s="20" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" ht="78.75" x14ac:dyDescent="0.25">
+      <c r="A8" s="13" t="s">
         <v>71</v>
       </c>
-      <c r="B7" s="14" t="s">
+      <c r="B8" s="14" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="8" spans="1:2" ht="54" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="13" t="s">
+    <row r="9" spans="1:2" ht="47.25" x14ac:dyDescent="0.25">
+      <c r="A9" s="13" t="s">
         <v>73</v>
       </c>
-      <c r="B8" s="14" t="s">
+      <c r="B9" s="14" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="9" spans="1:2" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="13" t="s">
+    <row r="10" spans="1:2" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A10" s="13" t="s">
         <v>75</v>
       </c>
-      <c r="B9" s="14" t="s">
+      <c r="B10" s="14" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="10" spans="1:2" ht="90" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="13" t="s">
+    <row r="11" spans="1:2" ht="94.5" x14ac:dyDescent="0.25">
+      <c r="A11" s="13" t="s">
         <v>76</v>
       </c>
-      <c r="B10" s="14" t="s">
+      <c r="B11" s="14" t="s">
         <v>77</v>
       </c>
     </row>

</xml_diff>